<commit_message>
Trim curation_benchmark to the manuscript pipeline; fix transcript selection to match the released database
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/curation_benchmark/results/supp_tables/supp_table_MWU.xlsx
+++ b/curation_benchmark/results/supp_tables/supp_table_MWU.xlsx
@@ -1,32 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ADRD (80%)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ASD (80%)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ASD_excl_ClinVar (80%)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="CHD (80%)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CHD_excl_ClinVar (80%)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="DDD (80%)" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="DDD_excl_ClinVar (80%)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Cancer_MSK (80%)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Cancer_TCGA (80%)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Cancer_AlphaMissense (80%)" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="ADRD (90%)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="ASD (90%)" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="ASD_excl_ClinVar (90%)" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="CHD (90%)" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="CHD_excl_ClinVar (90%)" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="DDD (90%)" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="DDD_excl_ClinVar (90%)" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Cancer_MSK (90%)" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Cancer_TCGA (90%)" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Cancer_AlphaMissense (90%)" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ADRD (80%)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASD (80%)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASD_excl_ClinVar (80%)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD (80%)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD_excl_ClinVar (80%)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DDD (80%)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DDD_excl_ClinVar (80%)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancer_MSK (80%)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancer_TCGA (80%)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancer_AlphaMissense (80%)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ADRD (90%)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASD (90%)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASD_excl_ClinVar (90%)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD (90%)" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CHD_excl_ClinVar (90%)" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DDD (90%)" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DDD_excl_ClinVar (90%)" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancer_MSK (90%)" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancer_TCGA (90%)" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cancer_AlphaMissense (90%)" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>